<commit_message>
Revision on scenario assumption for S1, S2, S3
</commit_message>
<xml_diff>
--- a/SType1.xlsx
+++ b/SType1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1_LASSO\LAS_Simulation_Jateng\I-O_Analysis\Regional-Economy---Jawa-Tengah\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6B4E44-69C6-4212-8E14-81D918116E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E9A316-7D4F-4557-90A2-9165B86689AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1EB512CF-4F19-4B5B-9369-4EA84374520F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1EB512CF-4F19-4B5B-9369-4EA84374520F}"/>
   </bookViews>
   <sheets>
     <sheet name="SType1" sheetId="1" r:id="rId1"/>
@@ -36,10 +36,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -486,10 +482,10 @@
     </row>
     <row r="4" spans="1:26">
       <c r="A4">
-        <v>7.0000000000000001E-3</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="B4">
-        <v>7.0000000000000001E-3</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -516,16 +512,16 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L4">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="O4">
         <v>0</v>
@@ -566,10 +562,10 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5">
-        <v>7.0000000000000001E-3</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="B5">
-        <v>7.0000000000000001E-3</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -886,10 +882,10 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9">
-        <v>7.0000000000000001E-3</v>
+        <v>0.05</v>
       </c>
       <c r="B9">
-        <v>7.0000000000000001E-3</v>
+        <v>0.05</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -928,13 +924,13 @@
         <v>0.5</v>
       </c>
       <c r="O9">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="P9">
         <v>0</v>
       </c>
       <c r="Q9">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="R9">
         <v>0</v>
@@ -966,10 +962,10 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10">
-        <v>7.0000000000000001E-3</v>
+        <v>0.05</v>
       </c>
       <c r="B10">
-        <v>7.0000000000000001E-3</v>
+        <v>0.05</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -1046,10 +1042,10 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1183,7 +1179,7 @@
         <v>0</v>
       </c>
       <c r="T12">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="U12">
         <v>0</v>
@@ -1286,10 +1282,10 @@
     </row>
     <row r="14" spans="1:26">
       <c r="A14">
-        <v>7.0000000000000001E-3</v>
+        <v>0.1</v>
       </c>
       <c r="B14">
-        <v>7.0000000000000001E-3</v>
+        <v>0.1</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1331,7 +1327,7 @@
         <v>0.1</v>
       </c>
       <c r="P14">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="Q14">
         <v>0</v>
@@ -1372,13 +1368,13 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -1515,13 +1511,13 @@
         <v>1</v>
       </c>
       <c r="X16">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="Y16">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="Z16">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="17" spans="1:26">
@@ -5526,10 +5522,10 @@
     </row>
     <row r="67" spans="1:26">
       <c r="A67">
-        <v>0.99</v>
+        <v>0.61</v>
       </c>
       <c r="B67">
-        <v>0.99399999999999999</v>
+        <v>0.61</v>
       </c>
       <c r="C67">
         <v>1</v>
@@ -5556,25 +5552,25 @@
         <v>0</v>
       </c>
       <c r="K67">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L67">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="M67">
-        <v>0.30000000000000004</v>
+        <v>0</v>
       </c>
       <c r="N67">
-        <v>0.30000000000000004</v>
+        <v>0</v>
       </c>
       <c r="O67">
-        <v>0.30000000000000004</v>
+        <v>0</v>
       </c>
       <c r="P67">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="Q67">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R67">
         <v>0</v>
@@ -5583,7 +5579,7 @@
         <v>0</v>
       </c>
       <c r="T67">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="U67">
         <v>1</v>
@@ -5595,13 +5591,13 @@
         <v>0</v>
       </c>
       <c r="X67">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="Y67">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="Z67">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
surplus, income, serapan tk
</commit_message>
<xml_diff>
--- a/SType1.xlsx
+++ b/SType1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1_LASSO\LAS_Simulation_Jateng\I-O_Analysis\Regional-Economy---Jawa-Tengah\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy---Jawa-Tengah/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E9A316-7D4F-4557-90A2-9165B86689AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{C2E9A316-7D4F-4557-90A2-9165B86689AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{124A6E68-EE02-413D-B785-4902235D2F95}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1EB512CF-4F19-4B5B-9369-4EA84374520F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1EB512CF-4F19-4B5B-9369-4EA84374520F}"/>
   </bookViews>
   <sheets>
     <sheet name="SType1" sheetId="1" r:id="rId1"/>
@@ -238,7 +238,7 @@
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:Z67"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
     <row r="1" spans="1:26">
       <c r="A1">
@@ -5528,13 +5528,13 @@
         <v>0.61</v>
       </c>
       <c r="C67">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="D67">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F67">
         <v>0</v>

</xml_diff>